<commit_message>
ANW-1860 Follow up: consolidate templates
</commit_message>
<xml_diff>
--- a/frontend/public/bulk_import_templates/bulk_import_template.xlsx
+++ b/frontend/public/bulk_import_templates/bulk_import_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zeffmorgan/src/lyrasis/archivesspace/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D71783-F4B3-4846-9F94-907FE5F5F64A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B037063-3885-AD41-A1FB-86137D1EC3A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34560" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="767" uniqueCount="505">
   <si>
     <t>This is the template for importing archival objects using the bulk_import ("Load SpreadSheet").  You may replace this line with something of your choosing after you've copied the file for your use.</t>
   </si>
@@ -1540,6 +1540,18 @@
   </si>
   <si>
     <t>Access Restrictions Type(1)</t>
+  </si>
+  <si>
+    <t>b_userestrict</t>
+  </si>
+  <si>
+    <t>e_userestrict</t>
+  </si>
+  <si>
+    <t>Use Restrictions Begin Date</t>
+  </si>
+  <si>
+    <t>Use Restrictions End Date</t>
   </si>
 </sst>
 </file>
@@ -2353,7 +2365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMJ1005"/>
+  <dimension ref="A1:AML1005"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.1640625" style="1" customWidth="1"/>
@@ -2495,10 +2507,10 @@
     <col min="178" max="178" width="10.1640625" style="2" customWidth="1"/>
     <col min="179" max="179" width="17.6640625" style="2" customWidth="1"/>
     <col min="180" max="180" width="17.6640625" customWidth="1"/>
-    <col min="181" max="1024" width="9.33203125" style="2"/>
+    <col min="181" max="1026" width="9.33203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2520,7 +2532,7 @@
       <c r="FU1" s="2"/>
       <c r="FX1" s="2"/>
     </row>
-    <row r="2" spans="1:188" ht="60" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:190" ht="60" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -3082,8 +3094,14 @@
       <c r="GE2" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:188" ht="105.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="GF2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="GG2" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:190" ht="105.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="19" t="s">
         <v>15</v>
       </c>
@@ -3643,8 +3661,14 @@
       <c r="GE3" s="36" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="4" spans="1:188" s="43" customFormat="1" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="GF3" s="36" t="s">
+        <v>503</v>
+      </c>
+      <c r="GG3" s="36" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="4" spans="1:190" s="43" customFormat="1" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="37" t="s">
         <v>151</v>
       </c>
@@ -4206,9 +4230,15 @@
       <c r="GE4" s="38" t="s">
         <v>335</v>
       </c>
-      <c r="GF4" s="2"/>
-    </row>
-    <row r="5" spans="1:188" ht="57" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="GF4" s="38" t="s">
+        <v>501</v>
+      </c>
+      <c r="GG4" s="38" t="s">
+        <v>502</v>
+      </c>
+      <c r="GH4" s="2"/>
+    </row>
+    <row r="5" spans="1:190" ht="57" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="44" t="s">
         <v>336</v>
       </c>
@@ -4770,13 +4800,19 @@
       <c r="GE5" s="47" t="s">
         <v>150</v>
       </c>
-      <c r="GF5" s="43"/>
-    </row>
-    <row r="6" spans="1:188" x14ac:dyDescent="0.2">
+      <c r="GF5" s="47" t="s">
+        <v>503</v>
+      </c>
+      <c r="GG5" s="47" t="s">
+        <v>504</v>
+      </c>
+      <c r="GH5" s="43"/>
+    </row>
+    <row r="6" spans="1:190" x14ac:dyDescent="0.2">
       <c r="BM6" s="51"/>
       <c r="BN6" s="2"/>
     </row>
-    <row r="7" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY7" s="2"/>
       <c r="EB7" s="2"/>
       <c r="EH7" s="2"/>
@@ -4796,7 +4832,7 @@
       <c r="FU7" s="2"/>
       <c r="FX7" s="2"/>
     </row>
-    <row r="8" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY8" s="2"/>
       <c r="EB8" s="2"/>
       <c r="EH8" s="2"/>
@@ -4816,7 +4852,7 @@
       <c r="FU8" s="2"/>
       <c r="FX8" s="2"/>
     </row>
-    <row r="9" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY9" s="2"/>
       <c r="EB9" s="2"/>
       <c r="EH9" s="2"/>
@@ -4836,7 +4872,7 @@
       <c r="FU9" s="2"/>
       <c r="FX9" s="2"/>
     </row>
-    <row r="10" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY10" s="2"/>
       <c r="EB10" s="2"/>
       <c r="EH10" s="2"/>
@@ -4856,7 +4892,7 @@
       <c r="FU10" s="2"/>
       <c r="FX10" s="2"/>
     </row>
-    <row r="11" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY11" s="2"/>
       <c r="EB11" s="2"/>
       <c r="EH11" s="2"/>
@@ -4876,7 +4912,7 @@
       <c r="FU11" s="2"/>
       <c r="FX11" s="2"/>
     </row>
-    <row r="12" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY12" s="2"/>
       <c r="EB12" s="2"/>
       <c r="EH12" s="2"/>
@@ -4896,7 +4932,7 @@
       <c r="FU12" s="2"/>
       <c r="FX12" s="2"/>
     </row>
-    <row r="13" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY13" s="2"/>
       <c r="EB13" s="2"/>
       <c r="EH13" s="2"/>
@@ -4916,7 +4952,7 @@
       <c r="FU13" s="2"/>
       <c r="FX13" s="2"/>
     </row>
-    <row r="14" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY14" s="2"/>
       <c r="EB14" s="2"/>
       <c r="EH14" s="2"/>
@@ -4936,7 +4972,7 @@
       <c r="FU14" s="2"/>
       <c r="FX14" s="2"/>
     </row>
-    <row r="15" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY15" s="2"/>
       <c r="EB15" s="2"/>
       <c r="EH15" s="2"/>
@@ -4956,7 +4992,7 @@
       <c r="FU15" s="2"/>
       <c r="FX15" s="2"/>
     </row>
-    <row r="16" spans="1:188" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:190" x14ac:dyDescent="0.2">
       <c r="DY16" s="2"/>
       <c r="EB16" s="2"/>
       <c r="EH16" s="2"/>
@@ -24757,7 +24793,7 @@
       <c r="FX1005" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="10">
+  <dataValidations disablePrompts="1" count="10">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I6:I1005" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Class,Collection,File,Fonds,Item,Other Level,Record Group,Series,Sub-Fonds,Sub-Group,Sub-Series"</formula1>
       <formula2>0</formula2>
@@ -24790,7 +24826,7 @@
       <formula1>"Creator,Source,Subject"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU6:BU7 CF6 BU8:BU1005" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF6 BU6:BU1005" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"MD5,SHA-1,SHA-256,SHA-384,SHA-512"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
ANW-1866 update spec and template documentation
</commit_message>
<xml_diff>
--- a/frontend/public/bulk_import_templates/bulk_import_template.xlsx
+++ b/frontend/public/bulk_import_templates/bulk_import_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zeffmorgan/src/lyrasis/archivesspace/frontend/public/bulk_import_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95EC3F3-3BEC-0B42-BF65-4C58D83A38D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F8A5BC-475F-9642-9BC6-1B5C95CE886A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34560" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="514">
   <si>
     <t>This is the template for importing archival objects using the bulk_import ("Load SpreadSheet").  You may replace this line with something of your choosing after you've copied the file for your use.</t>
   </si>
@@ -1495,9 +1495,6 @@
   </si>
   <si>
     <t>Ref_ids will be generated for Archival Objects and Digital Objects created with this process.</t>
-  </si>
-  <si>
-    <t>Date Era and Calendar will be set to blank during import.</t>
   </si>
   <si>
     <t xml:space="preserve">barcode will not be added to an existing top container. </t>
@@ -2630,28 +2627,28 @@
         <v>5</v>
       </c>
       <c r="V2" s="10" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="W2" s="10" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="X2" s="10" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="Y2" s="10" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="Z2" s="10" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AA2" s="10" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AB2" s="10" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AC2" s="10" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AD2" s="10" t="s">
         <v>6</v>
@@ -3227,10 +3224,10 @@
         <v>39</v>
       </c>
       <c r="AB3" s="25" t="s">
+        <v>499</v>
+      </c>
+      <c r="AC3" s="25" t="s">
         <v>500</v>
-      </c>
-      <c r="AC3" s="25" t="s">
-        <v>501</v>
       </c>
       <c r="AD3" s="24" t="s">
         <v>34</v>
@@ -3251,10 +3248,10 @@
         <v>39</v>
       </c>
       <c r="AJ3" s="25" t="s">
+        <v>499</v>
+      </c>
+      <c r="AK3" s="25" t="s">
         <v>500</v>
-      </c>
-      <c r="AK3" s="25" t="s">
-        <v>501</v>
       </c>
       <c r="AL3" s="27" t="s">
         <v>40</v>
@@ -3719,10 +3716,10 @@
         <v>149</v>
       </c>
       <c r="GJ3" s="36" t="s">
+        <v>510</v>
+      </c>
+      <c r="GK3" s="36" t="s">
         <v>511</v>
-      </c>
-      <c r="GK3" s="36" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="4" spans="1:193" s="43" customFormat="1" ht="56.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -3790,28 +3787,28 @@
         <v>170</v>
       </c>
       <c r="V4" s="38" t="s">
+        <v>493</v>
+      </c>
+      <c r="W4" s="39" t="s">
         <v>494</v>
       </c>
-      <c r="W4" s="39" t="s">
+      <c r="X4" s="39" t="s">
         <v>495</v>
       </c>
-      <c r="X4" s="39" t="s">
+      <c r="Y4" s="38" t="s">
         <v>496</v>
       </c>
-      <c r="Y4" s="38" t="s">
+      <c r="Z4" s="39" t="s">
         <v>497</v>
       </c>
-      <c r="Z4" s="39" t="s">
+      <c r="AA4" s="38" t="s">
         <v>498</v>
       </c>
-      <c r="AA4" s="38" t="s">
-        <v>499</v>
-      </c>
       <c r="AB4" s="39" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="AC4" s="39" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AD4" s="38" t="s">
         <v>171</v>
@@ -3832,10 +3829,10 @@
         <v>176</v>
       </c>
       <c r="AJ4" s="39" t="s">
+        <v>506</v>
+      </c>
+      <c r="AK4" s="39" t="s">
         <v>507</v>
-      </c>
-      <c r="AK4" s="39" t="s">
-        <v>508</v>
       </c>
       <c r="AL4" s="38" t="s">
         <v>177</v>
@@ -4162,7 +4159,7 @@
         <v>283</v>
       </c>
       <c r="EP4" s="38" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="EQ4" s="40" t="s">
         <v>284</v>
@@ -4300,10 +4297,10 @@
         <v>328</v>
       </c>
       <c r="GJ4" s="38" t="s">
+        <v>512</v>
+      </c>
+      <c r="GK4" s="38" t="s">
         <v>513</v>
-      </c>
-      <c r="GK4" s="38" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="5" spans="1:193" ht="57" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -4389,10 +4386,10 @@
         <v>351</v>
       </c>
       <c r="AB5" s="50" t="s">
+        <v>502</v>
+      </c>
+      <c r="AC5" s="50" t="s">
         <v>503</v>
-      </c>
-      <c r="AC5" s="50" t="s">
-        <v>504</v>
       </c>
       <c r="AD5" s="47" t="s">
         <v>352</v>
@@ -4413,10 +4410,10 @@
         <v>357</v>
       </c>
       <c r="AJ5" s="50" t="s">
+        <v>508</v>
+      </c>
+      <c r="AK5" s="50" t="s">
         <v>509</v>
-      </c>
-      <c r="AK5" s="50" t="s">
-        <v>510</v>
       </c>
       <c r="AL5" s="47" t="s">
         <v>358</v>
@@ -4743,7 +4740,7 @@
         <v>451</v>
       </c>
       <c r="EP5" s="47" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="EQ5" s="47" t="s">
         <v>452</v>
@@ -4881,10 +4878,10 @@
         <v>149</v>
       </c>
       <c r="GJ5" s="47" t="s">
+        <v>510</v>
+      </c>
+      <c r="GK5" s="47" t="s">
         <v>511</v>
-      </c>
-      <c r="GK5" s="47" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="6" spans="1:193" ht="16" thickTop="1" x14ac:dyDescent="0.2">
@@ -24921,7 +24918,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="128.33203125" customWidth="1"/>
@@ -24960,11 +24957,6 @@
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>487</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>488</v>
       </c>
     </row>
   </sheetData>
@@ -24983,17 +24975,17 @@
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
   </sheetData>

</xml_diff>